<commit_message>
dados atualizados com os dados COPOM
</commit_message>
<xml_diff>
--- a/R Markdown/resultados/df_ciclo_2022_2025.xlsx
+++ b/R Markdown/resultados/df_ciclo_2022_2025.xlsx
@@ -426,7 +426,7 @@
         <v>0.01278087722546964</v>
       </c>
       <c r="C2">
-        <v>268083860.93</v>
+        <v>270800600.28</v>
       </c>
       <c r="D2">
         <v>600441154.33</v>
@@ -435,19 +435,19 @@
         <v>737074530.21</v>
       </c>
       <c r="F2">
-        <v>985402150.88</v>
+        <v>989484961.0599999</v>
       </c>
       <c r="G2">
-        <v>2591001696.35</v>
+        <v>2597801245.88</v>
       </c>
       <c r="H2">
-        <v>0.01706572090368024</v>
+        <v>0.01706066772054106</v>
       </c>
       <c r="I2">
-        <v>0.004284843678210599</v>
+        <v>0.004279790495071413</v>
       </c>
       <c r="J2">
-        <v>0.3352542710974324</v>
+        <v>0.3348589004941442</v>
       </c>
       <c r="K2" t="inlineStr">
         <is>
@@ -470,7 +470,7 @@
         <v>0.03138103348631988</v>
       </c>
       <c r="C3">
-        <v>529830929.79</v>
+        <v>531726447.48</v>
       </c>
       <c r="D3">
         <v>1086938304.9</v>
@@ -479,19 +479,19 @@
         <v>1370494139.28</v>
       </c>
       <c r="F3">
-        <v>2112006389.73</v>
+        <v>2120033849.32</v>
       </c>
       <c r="G3">
-        <v>5099269763.700001</v>
+        <v>5109192740.98</v>
       </c>
       <c r="H3">
-        <v>0.03358651394264638</v>
+        <v>0.03355385244052139</v>
       </c>
       <c r="I3">
-        <v>0.002205480456326507</v>
+        <v>0.002172818954201516</v>
       </c>
       <c r="J3">
-        <v>0.07028068267056774</v>
+        <v>0.06923987876781452</v>
       </c>
       <c r="K3" t="inlineStr">
         <is>
@@ -514,7 +514,7 @@
         <v>0.07049848664210395</v>
       </c>
       <c r="C4">
-        <v>1135615346.88</v>
+        <v>1136043087.37</v>
       </c>
       <c r="D4">
         <v>1893010845.67</v>
@@ -523,19 +523,19 @@
         <v>1802521652.49</v>
       </c>
       <c r="F4">
-        <v>2560599212.5</v>
+        <v>2562583888.81</v>
       </c>
       <c r="G4">
-        <v>7391747057.54</v>
+        <v>7394159474.34</v>
       </c>
       <c r="H4">
-        <v>0.04868599370362481</v>
+        <v>0.04856002670122379</v>
       </c>
       <c r="I4">
-        <v>-0.02181249293847914</v>
+        <v>-0.02193845994088016</v>
       </c>
       <c r="J4">
-        <v>-0.309403704638562</v>
+        <v>-0.311190508985732</v>
       </c>
       <c r="K4" t="inlineStr">
         <is>
@@ -558,7 +558,7 @@
         <v>0.08227494643576272</v>
       </c>
       <c r="C5">
-        <v>901971023.1900001</v>
+        <v>903229166.3</v>
       </c>
       <c r="D5">
         <v>1726163460.9</v>
@@ -567,19 +567,19 @@
         <v>2114329482</v>
       </c>
       <c r="F5">
-        <v>3213515525.28</v>
+        <v>3217471932.62</v>
       </c>
       <c r="G5">
-        <v>7955979491.370001</v>
+        <v>7961194041.82</v>
       </c>
       <c r="H5">
-        <v>0.0524023298426986</v>
+        <v>0.05228394066776743</v>
       </c>
       <c r="I5">
-        <v>-0.02987261659306412</v>
+        <v>-0.02999100576799529</v>
       </c>
       <c r="J5">
-        <v>-0.363082783850702</v>
+        <v>-0.3645217294843354</v>
       </c>
       <c r="K5" t="inlineStr">
         <is>
@@ -602,7 +602,7 @@
         <v>0.02290605900133662</v>
       </c>
       <c r="C6">
-        <v>154312005.2</v>
+        <v>156688314.62</v>
       </c>
       <c r="D6">
         <v>842834351.62</v>
@@ -611,19 +611,19 @@
         <v>745939592.83</v>
       </c>
       <c r="F6">
-        <v>989313791.46</v>
+        <v>990146048.22</v>
       </c>
       <c r="G6">
-        <v>2732399741.11</v>
+        <v>2735608307.29</v>
       </c>
       <c r="H6">
-        <v>0.01799704394048086</v>
+        <v>0.01796569480372878</v>
       </c>
       <c r="I6">
-        <v>-0.004909015060855754</v>
+        <v>-0.004940364197607842</v>
       </c>
       <c r="J6">
-        <v>-0.2143107664469607</v>
+        <v>-0.2156793622735173</v>
       </c>
       <c r="K6" t="inlineStr">
         <is>
@@ -646,7 +646,7 @@
         <v>0.05427611013661751</v>
       </c>
       <c r="C7">
-        <v>530860636.58</v>
+        <v>530941174.36</v>
       </c>
       <c r="D7">
         <v>1031792894.37</v>
@@ -655,19 +655,19 @@
         <v>1014230423.52</v>
       </c>
       <c r="F7">
-        <v>1687158182.77</v>
+        <v>1688434491</v>
       </c>
       <c r="G7">
-        <v>4264042137.24</v>
+        <v>4265398983.25</v>
       </c>
       <c r="H7">
-        <v>0.02808525873919003</v>
+        <v>0.02801236425002599</v>
       </c>
       <c r="I7">
-        <v>-0.02619085139742748</v>
+        <v>-0.02626374588659152</v>
       </c>
       <c r="J7">
-        <v>-0.4825484238185624</v>
+        <v>-0.4838914546470532</v>
       </c>
       <c r="K7" t="inlineStr">
         <is>
@@ -690,7 +690,7 @@
         <v>0.02476472440077774</v>
       </c>
       <c r="C8">
-        <v>318218981.72</v>
+        <v>323404422.56</v>
       </c>
       <c r="D8">
         <v>434812479.76</v>
@@ -702,16 +702,16 @@
         <v>1335237845.73</v>
       </c>
       <c r="G8">
-        <v>2990942599.59</v>
+        <v>2996128040.43</v>
       </c>
       <c r="H8">
-        <v>0.01969994528194852</v>
+        <v>0.01967661884335443</v>
       </c>
       <c r="I8">
-        <v>-0.005064779118829223</v>
+        <v>-0.005088105557423311</v>
       </c>
       <c r="J8">
-        <v>-0.2045158684935804</v>
+        <v>-0.2054577904878085</v>
       </c>
       <c r="K8" t="inlineStr">
         <is>
@@ -734,7 +734,7 @@
         <v>0.01564514619986043</v>
       </c>
       <c r="C9">
-        <v>299824744.02</v>
+        <v>300184054.28</v>
       </c>
       <c r="D9">
         <v>419672736.3</v>
@@ -743,19 +743,19 @@
         <v>500741801.08</v>
       </c>
       <c r="F9">
-        <v>1133248138.6</v>
+        <v>1144062973.34</v>
       </c>
       <c r="G9">
-        <v>2353487420</v>
+        <v>2364661565</v>
       </c>
       <c r="H9">
-        <v>0.01550132503449238</v>
+        <v>0.01552955804297244</v>
       </c>
       <c r="I9">
-        <v>-0.0001438211653680532</v>
+        <v>-0.0001155881568879885</v>
       </c>
       <c r="J9">
-        <v>-0.009192701910918298</v>
+        <v>-0.007388116123134705</v>
       </c>
       <c r="K9" t="inlineStr">
         <is>
@@ -778,7 +778,7 @@
         <v>0.04493881006046815</v>
       </c>
       <c r="C10">
-        <v>658113599.2</v>
+        <v>662096967.22</v>
       </c>
       <c r="D10">
         <v>843947046.97</v>
@@ -787,19 +787,19 @@
         <v>1100647553.21</v>
       </c>
       <c r="F10">
-        <v>2299120389.61</v>
+        <v>2301085241.03</v>
       </c>
       <c r="G10">
-        <v>4901828588.99</v>
+        <v>4907776808.43</v>
       </c>
       <c r="H10">
-        <v>0.03228606092200873</v>
+        <v>0.03223108369356346</v>
       </c>
       <c r="I10">
-        <v>-0.01265274913845942</v>
+        <v>-0.01270772636690469</v>
       </c>
       <c r="J10">
-        <v>-0.2815550550055576</v>
+        <v>-0.2827784347161307</v>
       </c>
       <c r="K10" t="inlineStr">
         <is>
@@ -822,7 +822,7 @@
         <v>0.03106350078710079</v>
       </c>
       <c r="C11">
-        <v>516585406.56</v>
+        <v>515288534.05</v>
       </c>
       <c r="D11">
         <v>686451804.38</v>
@@ -831,19 +831,19 @@
         <v>920953728.14</v>
       </c>
       <c r="F11">
-        <v>1000682748.19</v>
+        <v>1001849833.82</v>
       </c>
       <c r="G11">
-        <v>3124673687.27</v>
+        <v>3124543900.39</v>
       </c>
       <c r="H11">
-        <v>0.02058076964486093</v>
+        <v>0.02051997062798372</v>
       </c>
       <c r="I11">
-        <v>-0.01048273114223986</v>
+        <v>-0.01054353015911707</v>
       </c>
       <c r="J11">
-        <v>-0.3374613574331211</v>
+        <v>-0.3394186067880443</v>
       </c>
       <c r="K11" t="inlineStr">
         <is>
@@ -866,7 +866,7 @@
         <v>0.02852737800077722</v>
       </c>
       <c r="C12">
-        <v>583297851.04</v>
+        <v>585362030.52</v>
       </c>
       <c r="D12">
         <v>1081771738.47</v>
@@ -875,19 +875,19 @@
         <v>1187638555.17</v>
       </c>
       <c r="F12">
-        <v>1586731172.63</v>
+        <v>1586731737.63</v>
       </c>
       <c r="G12">
-        <v>4439439317.31</v>
+        <v>4441504061.79</v>
       </c>
       <c r="H12">
-        <v>0.02924051823847321</v>
+        <v>0.02916890778222873</v>
       </c>
       <c r="I12">
-        <v>0.0007131402376959924</v>
+        <v>0.0006415297814515129</v>
       </c>
       <c r="J12">
-        <v>0.02499845017921251</v>
+        <v>0.022488214003896</v>
       </c>
       <c r="K12" t="inlineStr">
         <is>
@@ -910,7 +910,7 @@
         <v>0.03440060917127755</v>
       </c>
       <c r="C13">
-        <v>677605266.5599999</v>
+        <v>677606342.2</v>
       </c>
       <c r="D13">
         <v>729781207.34</v>
@@ -919,19 +919,19 @@
         <v>809483850.37</v>
       </c>
       <c r="F13">
-        <v>1202045954.4</v>
+        <v>1202924802.61</v>
       </c>
       <c r="G13">
-        <v>3418916278.67</v>
+        <v>3419796202.52</v>
       </c>
       <c r="H13">
-        <v>0.02251880849287939</v>
+        <v>0.02245899557392733</v>
       </c>
       <c r="I13">
-        <v>-0.01188180067839816</v>
+        <v>-0.01194161359735021</v>
       </c>
       <c r="J13">
-        <v>-0.3453950660943165</v>
+        <v>-0.347133782948261</v>
       </c>
       <c r="K13" t="inlineStr">
         <is>
@@ -954,7 +954,7 @@
         <v>0.04982071041328871</v>
       </c>
       <c r="C14">
-        <v>880773966.36</v>
+        <v>892661593.1899999</v>
       </c>
       <c r="D14">
         <v>1104357795.92</v>
@@ -963,19 +963,19 @@
         <v>1381059096.62</v>
       </c>
       <c r="F14">
-        <v>2038715032.19</v>
+        <v>2039768606.41</v>
       </c>
       <c r="G14">
-        <v>5404905891.09</v>
+        <v>5417847092.14</v>
       </c>
       <c r="H14">
-        <v>0.03559959670344393</v>
+        <v>0.03558089332133988</v>
       </c>
       <c r="I14">
-        <v>-0.01422111370984477</v>
+        <v>-0.01423981709194883</v>
       </c>
       <c r="J14">
-        <v>-0.2854458234712681</v>
+        <v>-0.2858212372690421</v>
       </c>
       <c r="K14" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
         <v>0.0146420577822676</v>
       </c>
       <c r="C15">
-        <v>288635829.29</v>
+        <v>289068585.26</v>
       </c>
       <c r="D15">
         <v>1149596326.06</v>
@@ -1007,19 +1007,19 @@
         <v>1278748563.6</v>
       </c>
       <c r="F15">
-        <v>1532409954.11</v>
+        <v>1532982112.9</v>
       </c>
       <c r="G15">
-        <v>4249390673.059999</v>
+        <v>4250395587.82</v>
       </c>
       <c r="H15">
-        <v>0.02798875637144617</v>
+        <v>0.02791383171428368</v>
       </c>
       <c r="I15">
-        <v>0.01334669858917857</v>
+        <v>0.01327177393201608</v>
       </c>
       <c r="J15">
-        <v>0.9115316158185236</v>
+        <v>0.9064145306193908</v>
       </c>
       <c r="K15" t="inlineStr">
         <is>
@@ -1042,7 +1042,7 @@
         <v>0.03619588619759224</v>
       </c>
       <c r="C16">
-        <v>417194492.06</v>
+        <v>418653600.77</v>
       </c>
       <c r="D16">
         <v>716643418.8</v>
@@ -1054,16 +1054,16 @@
         <v>1078973096.78</v>
       </c>
       <c r="G16">
-        <v>3231109115.94</v>
+        <v>3232568224.65</v>
       </c>
       <c r="H16">
-        <v>0.02128181022021238</v>
+        <v>0.02122940407862152</v>
       </c>
       <c r="I16">
-        <v>-0.01491407597737986</v>
+        <v>-0.01496648211897071</v>
       </c>
       <c r="J16">
-        <v>-0.412037873474471</v>
+        <v>-0.4134857214786549</v>
       </c>
       <c r="K16" t="inlineStr">
         <is>
@@ -1086,7 +1086,7 @@
         <v>0.01196759457375883</v>
       </c>
       <c r="C17">
-        <v>438963711.58</v>
+        <v>439828459.44</v>
       </c>
       <c r="D17">
         <v>1105161010.6</v>
@@ -1095,19 +1095,19 @@
         <v>1270053924.95</v>
       </c>
       <c r="F17">
-        <v>1621677779.68</v>
+        <v>1635541987.13</v>
       </c>
       <c r="G17">
-        <v>4435856426.81</v>
+        <v>4450585382.12</v>
       </c>
       <c r="H17">
-        <v>0.02921691940818778</v>
+        <v>0.02922854798328708</v>
       </c>
       <c r="I17">
-        <v>0.01724932483442895</v>
+        <v>0.01726095340952825</v>
       </c>
       <c r="J17">
-        <v>1.441335995142356</v>
+        <v>1.442307667020747</v>
       </c>
       <c r="K17" t="inlineStr">
         <is>
@@ -1130,7 +1130,7 @@
         <v>0.0768001000600067</v>
       </c>
       <c r="C18">
-        <v>407347161.41</v>
+        <v>407603040.74</v>
       </c>
       <c r="D18">
         <v>1414739277.9</v>
@@ -1139,19 +1139,19 @@
         <v>1550313121.75</v>
       </c>
       <c r="F18">
-        <v>3031872611.37</v>
+        <v>3036975936.59</v>
       </c>
       <c r="G18">
-        <v>6404272172.43</v>
+        <v>6409631376.98</v>
       </c>
       <c r="H18">
-        <v>0.04218195674663604</v>
+        <v>0.04209428696950479</v>
       </c>
       <c r="I18">
-        <v>-0.03461814331337066</v>
+        <v>-0.03470581309050191</v>
       </c>
       <c r="J18">
-        <v>-0.450756487118145</v>
+        <v>-0.4518980191872797</v>
       </c>
       <c r="K18" t="inlineStr">
         <is>
@@ -1174,7 +1174,7 @@
         <v>0.01518693116727706</v>
       </c>
       <c r="C19">
-        <v>443362279.2</v>
+        <v>444011947.82</v>
       </c>
       <c r="D19">
         <v>1177863319.16</v>
@@ -1183,19 +1183,19 @@
         <v>1879548379.37</v>
       </c>
       <c r="F19">
-        <v>2415683562.03</v>
+        <v>2415839399.78</v>
       </c>
       <c r="G19">
-        <v>5916457539.76</v>
+        <v>5917263046.13</v>
       </c>
       <c r="H19">
-        <v>0.03896894905713704</v>
+        <v>0.03886073224622813</v>
       </c>
       <c r="I19">
-        <v>0.02378201788985998</v>
+        <v>0.02367380107895107</v>
       </c>
       <c r="J19">
-        <v>1.565952833255909</v>
+        <v>1.55882717964512</v>
       </c>
       <c r="K19" t="inlineStr">
         <is>
@@ -1218,7 +1218,7 @@
         <v>0.04188065349285796</v>
       </c>
       <c r="C20">
-        <v>254026720.87</v>
+        <v>254092379.92</v>
       </c>
       <c r="D20">
         <v>599141447.25</v>
@@ -1227,19 +1227,19 @@
         <v>891442908.4</v>
       </c>
       <c r="F20">
-        <v>1292475939.08</v>
+        <v>1294481417.88</v>
       </c>
       <c r="G20">
-        <v>3037087015.6</v>
+        <v>3039158153.45</v>
       </c>
       <c r="H20">
-        <v>0.02000387704934154</v>
+        <v>0.01995921261813833</v>
       </c>
       <c r="I20">
-        <v>-0.02187677644351642</v>
+        <v>-0.02192144087471963</v>
       </c>
       <c r="J20">
-        <v>-0.5223599590499975</v>
+        <v>-0.5234264283497382</v>
       </c>
       <c r="K20" t="inlineStr">
         <is>
@@ -1262,7 +1262,7 @@
         <v>0.03328667005479251</v>
       </c>
       <c r="C21">
-        <v>409432833.7</v>
+        <v>413735667.28</v>
       </c>
       <c r="D21">
         <v>1002662305.98</v>
@@ -1271,19 +1271,19 @@
         <v>1355941790.68</v>
       </c>
       <c r="F21">
-        <v>1702354442.56</v>
+        <v>1705356170.99</v>
       </c>
       <c r="G21">
-        <v>4470391372.92</v>
+        <v>4477695934.93</v>
       </c>
       <c r="H21">
-        <v>0.02944438500675035</v>
+        <v>0.02940659244836891</v>
       </c>
       <c r="I21">
-        <v>-0.003842285048042161</v>
+        <v>-0.003880077606423601</v>
       </c>
       <c r="J21">
-        <v>-0.1154301419071795</v>
+        <v>-0.1165655080558279</v>
       </c>
       <c r="K21" t="inlineStr">
         <is>
@@ -1306,7 +1306,7 @@
         <v>0.021319194803451</v>
       </c>
       <c r="C22">
-        <v>317894841.59</v>
+        <v>318856012.44</v>
       </c>
       <c r="D22">
         <v>378277168.48</v>
@@ -1315,19 +1315,19 @@
         <v>643891246.63</v>
       </c>
       <c r="F22">
-        <v>915880639.14</v>
+        <v>918890507.58</v>
       </c>
       <c r="G22">
-        <v>2255943895.84</v>
+        <v>2259914935.13</v>
       </c>
       <c r="H22">
-        <v>0.01485885129098963</v>
+        <v>0.01484165035569546</v>
       </c>
       <c r="I22">
-        <v>-0.006460343512461365</v>
+        <v>-0.006477544447755532</v>
       </c>
       <c r="J22">
-        <v>-0.3030294329603673</v>
+        <v>-0.3038362615227379</v>
       </c>
       <c r="K22" t="inlineStr">
         <is>
@@ -1350,7 +1350,7 @@
         <v>0.006306371387863901</v>
       </c>
       <c r="C23">
-        <v>176159856.34</v>
+        <v>179126600.35</v>
       </c>
       <c r="D23">
         <v>681661685.0599999</v>
@@ -1359,19 +1359,19 @@
         <v>623666594.01</v>
       </c>
       <c r="F23">
-        <v>996106805.3</v>
+        <v>997429393.05</v>
       </c>
       <c r="G23">
-        <v>2477594940.71</v>
+        <v>2481884272.47</v>
       </c>
       <c r="H23">
-        <v>0.0163187634458482</v>
+        <v>0.01629940048747031</v>
       </c>
       <c r="I23">
-        <v>0.0100123920579843</v>
+        <v>0.009993029099606409</v>
       </c>
       <c r="J23">
-        <v>1.587662927250421</v>
+        <v>1.584592546965626</v>
       </c>
       <c r="K23" t="inlineStr">
         <is>
@@ -1394,7 +1394,7 @@
         <v>0.03550998362496413</v>
       </c>
       <c r="C24">
-        <v>367540618.45</v>
+        <v>373444861.42</v>
       </c>
       <c r="D24">
         <v>624679391.73</v>
@@ -1403,19 +1403,19 @@
         <v>856333446.46</v>
       </c>
       <c r="F24">
-        <v>1780968666.97</v>
+        <v>1785675753.86</v>
       </c>
       <c r="G24">
-        <v>3629522123.61</v>
+        <v>3640133453.47</v>
       </c>
       <c r="H24">
-        <v>0.02390597106227984</v>
+        <v>0.02390602722458852</v>
       </c>
       <c r="I24">
-        <v>-0.01160401256268429</v>
+        <v>-0.01160395640037561</v>
       </c>
       <c r="J24">
-        <v>-0.3267816928681001</v>
+        <v>-0.3267801112760251</v>
       </c>
       <c r="K24" t="inlineStr">
         <is>
@@ -1438,7 +1438,7 @@
         <v>0.01442360309469943</v>
       </c>
       <c r="C25">
-        <v>165422674.2</v>
+        <v>166699640.05</v>
       </c>
       <c r="D25">
         <v>1743044894.91</v>
@@ -1447,19 +1447,19 @@
         <v>1554935421.67</v>
       </c>
       <c r="F25">
-        <v>1366325941.16</v>
+        <v>1376552981.17</v>
       </c>
       <c r="G25">
-        <v>4829728931.940001</v>
+        <v>4841232937.8</v>
       </c>
       <c r="H25">
-        <v>0.03181117407565904</v>
+        <v>0.03179406686348163</v>
       </c>
       <c r="I25">
-        <v>0.01738757098095961</v>
+        <v>0.0173704637687822</v>
       </c>
       <c r="J25">
-        <v>1.205494276762885</v>
+        <v>1.204308219987398</v>
       </c>
       <c r="K25" t="inlineStr">
         <is>
@@ -1482,7 +1482,7 @@
         <v>0.00780842708567104</v>
       </c>
       <c r="C26">
-        <v>213876408.05</v>
+        <v>214276208.71</v>
       </c>
       <c r="D26">
         <v>790575300.34</v>
@@ -1491,19 +1491,19 @@
         <v>849590055.38</v>
       </c>
       <c r="F26">
-        <v>1660301401.41</v>
+        <v>1665436605.22</v>
       </c>
       <c r="G26">
-        <v>3514343165.18</v>
+        <v>3519878169.65</v>
       </c>
       <c r="H26">
-        <v>0.02314734093042313</v>
+        <v>0.0231162687924736</v>
       </c>
       <c r="I26">
-        <v>0.01533891384475209</v>
+        <v>0.01530784170680256</v>
       </c>
       <c r="J26">
-        <v>1.964405081389563</v>
+        <v>1.960425773187205</v>
       </c>
       <c r="K26" t="inlineStr">
         <is>
@@ -1526,7 +1526,7 @@
         <v>0.02854078087441063</v>
       </c>
       <c r="C27">
-        <v>297747200.45</v>
+        <v>297798794.47</v>
       </c>
       <c r="D27">
         <v>746739859.46</v>
@@ -1535,19 +1535,19 @@
         <v>730973098.37</v>
       </c>
       <c r="F27">
-        <v>1077859469.28</v>
+        <v>1078636355.45</v>
       </c>
       <c r="G27">
-        <v>2853319627.56</v>
+        <v>2854148107.75</v>
       </c>
       <c r="H27">
-        <v>0.01879348689023556</v>
+        <v>0.01874418705771267</v>
       </c>
       <c r="I27">
-        <v>-0.009747293984175068</v>
+        <v>-0.009796593816697955</v>
       </c>
       <c r="J27">
-        <v>-0.3415216292457643</v>
+        <v>-0.3432489762563393</v>
       </c>
       <c r="K27" t="inlineStr">
         <is>
@@ -1570,7 +1570,7 @@
         <v>0.05776210461891745</v>
       </c>
       <c r="C28">
-        <v>607742680.01</v>
+        <v>609449214.6</v>
       </c>
       <c r="D28">
         <v>1096779160.03</v>
@@ -1579,19 +1579,19 @@
         <v>1424727936.6</v>
       </c>
       <c r="F28">
-        <v>1955065802.96</v>
+        <v>1956937590.38</v>
       </c>
       <c r="G28">
-        <v>5084315579.6</v>
+        <v>5087893901.610001</v>
       </c>
       <c r="H28">
-        <v>0.033488017699841</v>
+        <v>0.0334139755265731</v>
       </c>
       <c r="I28">
-        <v>-0.02427408691907645</v>
+        <v>-0.02434812909234436</v>
       </c>
       <c r="J28">
-        <v>-0.420242425015908</v>
+        <v>-0.4215242718903665</v>
       </c>
       <c r="K28" t="inlineStr">
         <is>
@@ -1614,7 +1614,7 @@
         <v>0.03997675152969091</v>
       </c>
       <c r="C29">
-        <v>451930234.72</v>
+        <v>451987454.6</v>
       </c>
       <c r="D29">
         <v>646056157.14</v>
@@ -1623,19 +1623,19 @@
         <v>757654983.4</v>
       </c>
       <c r="F29">
-        <v>1356017191.47</v>
+        <v>1362970185.21</v>
       </c>
       <c r="G29">
-        <v>3211658566.73</v>
+        <v>3218668780.35</v>
       </c>
       <c r="H29">
-        <v>0.02115369851549649</v>
+        <v>0.02113812157535899</v>
       </c>
       <c r="I29">
-        <v>-0.01882305301419442</v>
+        <v>-0.01883862995433193</v>
       </c>
       <c r="J29">
-        <v>-0.4708499889045375</v>
+        <v>-0.4712396388771206</v>
       </c>
       <c r="K29" t="inlineStr">
         <is>
@@ -1658,28 +1658,28 @@
         <v>0.01774539803593836</v>
       </c>
       <c r="C30">
-        <v>2362273524.69</v>
+        <v>2593261890.04</v>
       </c>
       <c r="D30">
-        <v>4671432106.78</v>
+        <v>4671432106.8</v>
       </c>
       <c r="E30">
         <v>11259293445.76</v>
       </c>
       <c r="F30">
-        <v>6783905505.23</v>
+        <v>6837566518.55</v>
       </c>
       <c r="G30">
-        <v>25076904582.46</v>
+        <v>25361553961.15</v>
       </c>
       <c r="H30">
-        <v>0.1651698859693348</v>
+        <v>0.1665581790346631</v>
       </c>
       <c r="I30">
-        <v>0.1474244879333964</v>
+        <v>0.1488127809987247</v>
       </c>
       <c r="J30">
-        <v>8.307758869923862</v>
+        <v>8.385992847122722</v>
       </c>
       <c r="K30" t="inlineStr">
         <is>
@@ -1702,7 +1702,7 @@
         <v>0.01471389456597418</v>
       </c>
       <c r="C31">
-        <v>310130761.22</v>
+        <v>310244568.84</v>
       </c>
       <c r="D31">
         <v>885501416.5700001</v>
@@ -1711,19 +1711,19 @@
         <v>1250274401.01</v>
       </c>
       <c r="F31">
-        <v>1589744832.47</v>
+        <v>1594437761.49</v>
       </c>
       <c r="G31">
-        <v>4035651411.27</v>
+        <v>4040458147.91</v>
       </c>
       <c r="H31">
-        <v>0.02658095544526181</v>
+        <v>0.02653509925348209</v>
       </c>
       <c r="I31">
-        <v>0.01186706087928762</v>
+        <v>0.0118212046875079</v>
       </c>
       <c r="J31">
-        <v>0.8065207227140357</v>
+        <v>0.8034041996497913</v>
       </c>
       <c r="K31" t="inlineStr">
         <is>
@@ -1746,7 +1746,7 @@
         <v>0.007949529934269608</v>
       </c>
       <c r="C32">
-        <v>268759034.4</v>
+        <v>270403481.87</v>
       </c>
       <c r="D32">
         <v>918101079.46</v>
@@ -1755,19 +1755,19 @@
         <v>1373080195.35</v>
       </c>
       <c r="F32">
-        <v>1934281944.28</v>
+        <v>1939351672.66</v>
       </c>
       <c r="G32">
-        <v>4494222253.49</v>
+        <v>4500936429.34</v>
       </c>
       <c r="H32">
-        <v>0.0296013479131311</v>
+        <v>0.02955922088883137</v>
       </c>
       <c r="I32">
-        <v>0.02165181797886149</v>
+        <v>0.02160969095456176</v>
       </c>
       <c r="J32">
-        <v>2.723660160775384</v>
+        <v>2.718360850671761</v>
       </c>
       <c r="K32" t="inlineStr">
         <is>
@@ -1790,7 +1790,7 @@
         <v>0.01470567515443555</v>
       </c>
       <c r="C33">
-        <v>190668608.27</v>
+        <v>190978482.88</v>
       </c>
       <c r="D33">
         <v>490592596.61</v>
@@ -1802,16 +1802,16 @@
         <v>776448481.35</v>
       </c>
       <c r="G33">
-        <v>1948516079.72</v>
+        <v>1948825954.33</v>
       </c>
       <c r="H33">
-        <v>0.01283396751136005</v>
+        <v>0.01279862041205837</v>
       </c>
       <c r="I33">
-        <v>-0.001871707643075505</v>
+        <v>-0.001907054742377181</v>
       </c>
       <c r="J33">
-        <v>-0.1272779130110838</v>
+        <v>-0.129681549629632</v>
       </c>
       <c r="K33" t="inlineStr">
         <is>

</xml_diff>